<commit_message>
feat(flight-control): Roll-only FBW PI-D, receiver filtering, CH5 calibration, and telemetry codec
- control: Roll-only PI-D control (Pitch PID completely deactivated for anti-stall safety, pitch remains 100% manual direct in all modes)
- control: implement CH5 Schmitt-trigger hysteresis and debounce for modes 1-3, roll assist / extremum seeking, soft throttle ceiling, and trimmed neutrals
- telemetry: update 61-byte packet codec with dynamic PID gains (pitch gains at 0.00), active flight modes, and Ground Station logging/buzzer support
- ground station: add buzzer feedback, tune_pid_sysid tool, and telemetry logger sync
- tests: add comprehensive test suites for CH5 decoding, buzzer, and FBW PID control logic (104 passing)
</commit_message>
<xml_diff>
--- a/Code/Battery_Monitor/voltage_sensor_analysis.xlsx
+++ b/Code/Battery_Monitor/voltage_sensor_analysis.xlsx
@@ -135,7 +135,7 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -166,7 +166,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="pt-PT"/>
         </a:p>
@@ -261,7 +261,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="pt-PT"/>
                 </a:p>
@@ -458,7 +458,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>
@@ -524,7 +524,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-PT"/>
           </a:p>

</xml_diff>